<commit_message>
refactor: direct webhook and single RabbitMQ consumer
</commit_message>
<xml_diff>
--- a/log_push.xlsx
+++ b/log_push.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -932,6 +932,259 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-09 12:49:56</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TRT19</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0001263-34.2025.5.19.0003</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>processo não encontrado.
+x</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-09 12:51:27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TRT19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0025800-57.1989.5.19.0003</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>o processo 0025800-57.1989.5.19.0003 já está cadastrado no push.
+x</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-16 11:55:22</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TRT5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0000008-86.2026.5.05.0038</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>não foi possível confirmar inserção</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-19 11:20:28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TRT7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0001757-96.2025.5.07.0013</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>processo não encontrado.
+x</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-19 11:21:56</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TRT7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>0001286-51.2023.5.07.0013</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>processo não encontrado.
+x</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:23:29</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>19</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0001251-20.2025.5.19.0003</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exceção não tratada: Message: Failed to decode response from marionette
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-20 16:25:02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TRT19</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0025800-57.1989.5.19.0003</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>o processo 0025800-57.1989.5.19.0003 já está cadastrado no push.
+x</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-25 13:06:39</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>19</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0000182-19.2026.5.19.0002</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exceção não tratada: Alert Text: Não foi possível encontrar o PJe Office.
+Message: Unexpected alert dialog detected. Performed handler "dismiss"
+Stacktrace:
+RemoteError@chrome://remote/content/shared/RemoteError.sys.mjs:8:8
+WebDriverError@chrome://remote/content/shared/webdriver/Errors.sys.mjs:202:5
+UnexpectedAlertOpenError@chrome://remote/content/shared/webdriver/Errors.sys.mjs:927:5
+GeckoDriver.prototype._handleUserPrompts@chrome://remote/content/marionette/driver.sys.mjs:3371:11
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-26 10:31:48</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TRT6</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0000236-33.2022.5.06.0019</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>o processo 0000236-33.2022.5.06.0019 já está cadastrado no push.
+x</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update: new template dashboard
</commit_message>
<xml_diff>
--- a/log_push.xlsx
+++ b/log_push.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1185,6 +1185,141 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-26 11:25:31</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>TRT6</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0000822-39.2023.5.06.0018</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>registro inserido (validação por total: 3904)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-26 11:27:22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TRT6</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0001057-41.2025.5.06.0016</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>registro inserido (validação por total: 3905)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-26 14:17:32</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TRT13</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0001184-20.2025.5.13.0004</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>registro inserido (validação por total: 895)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-26 14:44:28</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TRT19</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0000382-26.2026.5.19.0002</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>registro inserido (validação por total: 265)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-26 15:30:56</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TRT5</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0000596-06.2020.5.05.0038</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SUCESSO</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>registro inserido (validação por total: 170)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: persist status to SQLite from dedicated consumers
</commit_message>
<xml_diff>
--- a/log_push.xlsx
+++ b/log_push.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2478,6 +2478,56 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-06 18:20:28</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>13</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>0001281-88.2024.5.13.0025</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Erro interno na automacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-06 18:21:06</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>13</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>0021500-83.2013.5.13.0001</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Erro interno na automacao</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>